<commit_message>
Them thu muc Bao cao Tuan 2 va Tuan 3
</commit_message>
<xml_diff>
--- a/BaoCao_Tuan/Tuan_2/Phan_cong_nhiem_vu_tung_thanh_vien.xlsx
+++ b/BaoCao_Tuan/Tuan_2/Phan_cong_nhiem_vu_tung_thanh_vien.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dai_hoc\PhatTrienUngDungDIDong\ESP32_Fingerprint_Attendance\BaoCao_Tuan\Tuan_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7AB4811-487F-44D8-9F02-840C255B2E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF63DC0-362A-4F43-9B2F-5AFB53FECAAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="79">
   <si>
     <t>STT</t>
   </si>
@@ -269,9 +269,6 @@
   </si>
   <si>
     <t>5. Sheet 'Tổng quan' dùng để theo dõi nhanh khối lượng công việc của từng thành viên.</t>
-  </si>
-  <si>
-    <t>☑ Hoàn thành</t>
   </si>
 </sst>
 </file>
@@ -488,6 +485,15 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -499,15 +505,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -825,101 +822,99 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15">
+      <c r="A2" s="18">
         <v>1</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="19" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="19" t="s">
-        <v>79</v>
-      </c>
+      <c r="E2" s="15"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
       <c r="D3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="19"/>
+      <c r="E3" s="15"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
       <c r="D4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="19"/>
+      <c r="E4" s="15"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
       <c r="D5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="19"/>
+      <c r="E5" s="15"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
+      <c r="A6" s="18"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="20"/>
+      <c r="E6" s="16"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="21"/>
+      <c r="E7" s="17"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="19"/>
+      <c r="E8" s="15"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
       <c r="D9" s="4" t="s">
         <v>17</v>
       </c>
@@ -929,13 +924,13 @@
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17">
+      <c r="A10" s="20">
         <v>2</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="21" t="s">
         <v>19</v>
       </c>
       <c r="D10" s="5" t="s">
@@ -947,9 +942,9 @@
       <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
       <c r="D11" s="5" t="s">
         <v>21</v>
       </c>
@@ -959,9 +954,9 @@
       <c r="H11" s="5"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
       <c r="D12" s="5" t="s">
         <v>22</v>
       </c>
@@ -971,9 +966,9 @@
       <c r="H12" s="5"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
+      <c r="A13" s="20"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
       <c r="D13" s="5" t="s">
         <v>23</v>
       </c>
@@ -983,9 +978,9 @@
       <c r="H13" s="5"/>
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
       <c r="D14" s="5" t="s">
         <v>24</v>
       </c>
@@ -995,9 +990,9 @@
       <c r="H14" s="5"/>
     </row>
     <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
       <c r="D15" s="5" t="s">
         <v>25</v>
       </c>
@@ -1007,9 +1002,9 @@
       <c r="H15" s="5"/>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
       <c r="D16" s="5" t="s">
         <v>26</v>
       </c>
@@ -1019,9 +1014,9 @@
       <c r="H16" s="5"/>
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
+      <c r="A17" s="20"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
       <c r="D17" s="5" t="s">
         <v>27</v>
       </c>
@@ -1031,9 +1026,9 @@
       <c r="H17" s="5"/>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
       <c r="D18" s="5" t="s">
         <v>28</v>
       </c>
@@ -1043,9 +1038,9 @@
       <c r="H18" s="5"/>
     </row>
     <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
+      <c r="A19" s="20"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
       <c r="D19" s="5" t="s">
         <v>29</v>
       </c>
@@ -1055,57 +1050,51 @@
       <c r="H19" s="5"/>
     </row>
     <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
+      <c r="A20" s="18">
         <v>3</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="19" t="s">
         <v>31</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="4"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="15"/>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
       <c r="D21" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="4"/>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
       <c r="D22" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="4"/>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="15"/>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
       <c r="D23" s="4" t="s">
         <v>35</v>
       </c>
@@ -1115,9 +1104,9 @@
       <c r="H23" s="4"/>
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="15"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
       <c r="D24" s="4" t="s">
         <v>36</v>
       </c>
@@ -1127,9 +1116,9 @@
       <c r="H24" s="4"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15"/>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
       <c r="D25" s="4" t="s">
         <v>37</v>
       </c>
@@ -1139,9 +1128,9 @@
       <c r="H25" s="4"/>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
       <c r="D26" s="4" t="s">
         <v>38</v>
       </c>
@@ -1151,9 +1140,9 @@
       <c r="H26" s="4"/>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
       <c r="D27" s="4" t="s">
         <v>39</v>
       </c>
@@ -1163,9 +1152,9 @@
       <c r="H27" s="4"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
       <c r="D28" s="4" t="s">
         <v>40</v>
       </c>
@@ -1175,9 +1164,9 @@
       <c r="H28" s="4"/>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="15"/>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
       <c r="D29" s="4" t="s">
         <v>41</v>
       </c>
@@ -1187,43 +1176,39 @@
       <c r="H29" s="4"/>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="17">
+      <c r="A30" s="20">
         <v>4</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="21" t="s">
         <v>43</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>79</v>
-      </c>
+      <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="5"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="17"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
       <c r="D31" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>79</v>
-      </c>
+      <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="5"/>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="17"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
       <c r="D32" s="5" t="s">
         <v>46</v>
       </c>
@@ -1233,9 +1218,9 @@
       <c r="H32" s="5"/>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="17"/>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
+      <c r="A33" s="20"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
       <c r="D33" s="5" t="s">
         <v>47</v>
       </c>
@@ -1245,9 +1230,9 @@
       <c r="H33" s="5"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="17"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
       <c r="D34" s="5" t="s">
         <v>48</v>
       </c>
@@ -1257,9 +1242,9 @@
       <c r="H34" s="5"/>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="17"/>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
+      <c r="A35" s="20"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
       <c r="D35" s="5" t="s">
         <v>49</v>
       </c>
@@ -1269,9 +1254,9 @@
       <c r="H35" s="5"/>
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="17"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
+      <c r="A36" s="20"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
       <c r="D36" s="5" t="s">
         <v>50</v>
       </c>
@@ -1281,9 +1266,9 @@
       <c r="H36" s="5"/>
     </row>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="17"/>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
+      <c r="A37" s="20"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
       <c r="D37" s="5" t="s">
         <v>51</v>
       </c>
@@ -1293,9 +1278,9 @@
       <c r="H37" s="5"/>
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="17"/>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
+      <c r="A38" s="20"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
       <c r="D38" s="5" t="s">
         <v>52</v>
       </c>
@@ -1305,9 +1290,9 @@
       <c r="H38" s="5"/>
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="17"/>
-      <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
+      <c r="A39" s="20"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
       <c r="D39" s="5" t="s">
         <v>53</v>
       </c>
@@ -1317,29 +1302,27 @@
       <c r="H39" s="5"/>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="15">
+      <c r="A40" s="18">
         <v>5</v>
       </c>
-      <c r="B40" s="16" t="s">
+      <c r="B40" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C40" s="16" t="s">
+      <c r="C40" s="19" t="s">
         <v>55</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="E40" s="2"/>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="4"/>
     </row>
     <row r="41" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="15"/>
-      <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
       <c r="D41" s="4" t="s">
         <v>57</v>
       </c>
@@ -1349,9 +1332,9 @@
       <c r="H41" s="4"/>
     </row>
     <row r="42" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="15"/>
-      <c r="B42" s="15"/>
-      <c r="C42" s="15"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
       <c r="D42" s="4" t="s">
         <v>58</v>
       </c>
@@ -1361,9 +1344,9 @@
       <c r="H42" s="4"/>
     </row>
     <row r="43" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="15"/>
-      <c r="B43" s="15"/>
-      <c r="C43" s="15"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
       <c r="D43" s="4" t="s">
         <v>59</v>
       </c>
@@ -1373,9 +1356,9 @@
       <c r="H43" s="4"/>
     </row>
     <row r="44" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="15"/>
-      <c r="B44" s="15"/>
-      <c r="C44" s="15"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="18"/>
       <c r="D44" s="4" t="s">
         <v>60</v>
       </c>
@@ -1385,9 +1368,9 @@
       <c r="H44" s="4"/>
     </row>
     <row r="45" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="15"/>
-      <c r="B45" s="15"/>
-      <c r="C45" s="15"/>
+      <c r="A45" s="18"/>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
       <c r="D45" s="4" t="s">
         <v>61</v>
       </c>
@@ -1397,9 +1380,9 @@
       <c r="H45" s="4"/>
     </row>
     <row r="46" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
-      <c r="B46" s="15"/>
-      <c r="C46" s="15"/>
+      <c r="A46" s="18"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="18"/>
       <c r="D46" s="4" t="s">
         <v>62</v>
       </c>
@@ -1409,9 +1392,9 @@
       <c r="H46" s="4"/>
     </row>
     <row r="47" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="15"/>
-      <c r="B47" s="15"/>
-      <c r="C47" s="15"/>
+      <c r="A47" s="18"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
       <c r="D47" s="4" t="s">
         <v>63</v>
       </c>
@@ -1421,9 +1404,9 @@
       <c r="H47" s="4"/>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="15"/>
-      <c r="B48" s="15"/>
-      <c r="C48" s="15"/>
+      <c r="A48" s="18"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
       <c r="D48" s="4" t="s">
         <v>64</v>
       </c>
@@ -1433,9 +1416,9 @@
       <c r="H48" s="4"/>
     </row>
     <row r="49" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="15"/>
-      <c r="B49" s="15"/>
-      <c r="C49" s="15"/>
+      <c r="A49" s="18"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
       <c r="D49" s="4" t="s">
         <v>65</v>
       </c>
@@ -1445,9 +1428,9 @@
       <c r="H49" s="4"/>
     </row>
     <row r="50" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="15"/>
-      <c r="B50" s="15"/>
-      <c r="C50" s="15"/>
+      <c r="A50" s="18"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
       <c r="D50" s="4" t="s">
         <v>66</v>
       </c>
@@ -1459,6 +1442,12 @@
   </sheetData>
   <autoFilter ref="A1:H50" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="15">
+    <mergeCell ref="A2:A9"/>
+    <mergeCell ref="B2:B9"/>
+    <mergeCell ref="C2:C9"/>
+    <mergeCell ref="A10:A19"/>
+    <mergeCell ref="B10:B19"/>
+    <mergeCell ref="C10:C19"/>
     <mergeCell ref="A40:A50"/>
     <mergeCell ref="B40:B50"/>
     <mergeCell ref="C40:C50"/>
@@ -1468,12 +1457,6 @@
     <mergeCell ref="A30:A39"/>
     <mergeCell ref="B30:B39"/>
     <mergeCell ref="C30:C39"/>
-    <mergeCell ref="A2:A9"/>
-    <mergeCell ref="B2:B9"/>
-    <mergeCell ref="C2:C9"/>
-    <mergeCell ref="A10:A19"/>
-    <mergeCell ref="B10:B19"/>
-    <mergeCell ref="C10:C19"/>
   </mergeCells>
   <conditionalFormatting sqref="E2:E50">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">

</xml_diff>